<commit_message>
Suppression d'informations devenues superflues
</commit_message>
<xml_diff>
--- a/Lits d'hôpital 2020 à 2024.xlsx
+++ b/Lits d'hôpital 2020 à 2024.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://oxfamfrance-my.sharepoint.com/personal/rehl_oxfamfrance_org/Documents/Documents/Santé et climat/Données/Lits d'hôpital/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rehl\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="9" documentId="8_{E9A4C601-F31F-4C5C-B678-4D1BA4FC80B7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C5D55DAC-742C-42B4-9374-FECC93D194B0}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D41A6F1E-F775-4AA6-A1B2-B7E88D6C7785}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="33135" yWindow="2355" windowWidth="21600" windowHeight="11295" xr2:uid="{10C43AAE-C678-44DE-8120-0AD5489D527F}"/>
+    <workbookView xWindow="31590" yWindow="3885" windowWidth="21600" windowHeight="11295" xr2:uid="{10C43AAE-C678-44DE-8120-0AD5489D527F}"/>
   </bookViews>
   <sheets>
     <sheet name="Feuil1" sheetId="1" r:id="rId1"/>
@@ -36,12 +36,9 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3" uniqueCount="3">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2" uniqueCount="2">
   <si>
     <t>Annee</t>
-  </si>
-  <si>
-    <t>Température</t>
   </si>
   <si>
     <t>Nombre de lits d'hôpital</t>
@@ -51,19 +48,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="3">
-    <numFmt numFmtId="43" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
-    <numFmt numFmtId="164" formatCode="0.0"/>
+  <numFmts count="1">
     <numFmt numFmtId="165" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;??_-;_-@_-"/>
   </numFmts>
-  <fonts count="3" x14ac:knownFonts="1">
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Aptos Narrow"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -103,19 +91,15 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="164" fontId="2" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
-  <cellStyles count="2">
-    <cellStyle name="Milliers" xfId="1" builtinId="3"/>
+  <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -129,10 +113,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -452,293 +432,215 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B4927C64-54B7-4AE8-A67C-91D61C0F60CF}">
-  <dimension ref="A1:C26"/>
+  <dimension ref="A1:B26"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:3" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="3" t="s">
+    <row r="1" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="3" t="s">
-        <v>2</v>
-      </c>
-      <c r="C1" s="4" t="s">
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>2000</v>
       </c>
-      <c r="B2" s="2">
+      <c r="B2" s="1">
         <v>246826</v>
       </c>
-      <c r="C2" s="1">
-        <v>0.68758697072549024</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>2001</v>
       </c>
-      <c r="B3" s="2">
+      <c r="B3" s="1">
         <v>241927</v>
       </c>
-      <c r="C3" s="1">
-        <v>0.84578251072549027</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>2002</v>
       </c>
-      <c r="B4" s="2">
+      <c r="B4" s="1">
         <v>238378</v>
       </c>
-      <c r="C4" s="1">
-        <v>0.89996867072549025</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>2003</v>
       </c>
-      <c r="B5" s="2">
+      <c r="B5" s="1">
         <v>234129</v>
       </c>
-      <c r="C5" s="1">
-        <v>0.90067237072549033</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>2004</v>
       </c>
-      <c r="B6" s="2">
+      <c r="B6" s="1">
         <v>231592</v>
       </c>
-      <c r="C6" s="1">
-        <v>0.8238728907254903</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>2005</v>
       </c>
-      <c r="B7" s="2">
+      <c r="B7" s="1">
         <v>229932</v>
       </c>
-      <c r="C7" s="1">
-        <v>0.96336472072549029</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>2006</v>
       </c>
-      <c r="B8" s="2">
+      <c r="B8" s="1">
         <v>227677</v>
       </c>
-      <c r="C8" s="1">
-        <v>0.92905487072549031</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>2007</v>
       </c>
-      <c r="B9" s="2">
+      <c r="B9" s="1">
         <v>226484</v>
       </c>
-      <c r="C9" s="1">
-        <v>0.94820347072549027</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>2008</v>
       </c>
-      <c r="B10" s="2">
+      <c r="B10" s="1">
         <v>223467</v>
       </c>
-      <c r="C10" s="1">
-        <v>0.82215201072549027</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>2009</v>
       </c>
-      <c r="B11" s="2">
+      <c r="B11" s="1">
         <v>223270</v>
       </c>
-      <c r="C11" s="1">
-        <v>0.95328387072549026</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>2010</v>
       </c>
-      <c r="B12" s="2">
+      <c r="B12" s="1">
         <v>222418</v>
       </c>
-      <c r="C12" s="1">
-        <v>1.0368736307254904</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>2011</v>
       </c>
-      <c r="B13" s="2">
+      <c r="B13" s="1">
         <v>223324</v>
       </c>
-      <c r="C13" s="1">
-        <v>0.89419990072549027</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>2012</v>
       </c>
-      <c r="B14" s="2">
+      <c r="B14" s="1">
         <v>222031</v>
       </c>
-      <c r="C14" s="1">
-        <v>0.93410927072549033</v>
-      </c>
-    </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>2013</v>
       </c>
-      <c r="B15" s="2">
+      <c r="B15" s="1">
         <v>219694</v>
       </c>
-      <c r="C15" s="1">
-        <v>0.98007757072549029</v>
-      </c>
-    </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>2014</v>
       </c>
-      <c r="B16" s="2">
+      <c r="B16" s="1">
         <v>216686</v>
       </c>
-      <c r="C16" s="1">
-        <v>1.0293738207254903</v>
-      </c>
-    </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17">
         <v>2015</v>
       </c>
-      <c r="B17" s="2">
+      <c r="B17" s="1">
         <v>213560</v>
       </c>
-      <c r="C17" s="1">
-        <v>1.1816165407254902</v>
-      </c>
-    </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18">
         <v>2016</v>
       </c>
-      <c r="B18" s="2">
+      <c r="B18" s="1">
         <v>210110</v>
       </c>
-      <c r="C18" s="1">
-        <v>1.2894293007254904</v>
-      </c>
-    </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19">
         <v>2017</v>
       </c>
-      <c r="B19" s="2">
+      <c r="B19" s="1">
         <v>206294</v>
       </c>
-      <c r="C19" s="1">
-        <v>1.2016764207254904</v>
-      </c>
-    </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20">
         <v>2018</v>
       </c>
-      <c r="B20" s="2">
+      <c r="B20" s="1">
         <v>203670</v>
       </c>
-      <c r="C20" s="1">
-        <v>1.1191561707254905</v>
-      </c>
-    </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A21">
         <v>2019</v>
       </c>
-      <c r="B21" s="2">
+      <c r="B21" s="1">
         <v>201026</v>
       </c>
-      <c r="C21" s="1">
-        <v>1.2475747707254903</v>
-      </c>
-    </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A22">
         <v>2020</v>
       </c>
-      <c r="B22" s="2">
+      <c r="B22" s="1">
         <v>197705</v>
       </c>
-      <c r="C22" s="1">
-        <v>1.26</v>
-      </c>
-    </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A23">
         <v>2021</v>
       </c>
-      <c r="B23" s="2">
+      <c r="B23" s="1">
         <v>194158</v>
       </c>
-      <c r="C23" s="1">
-        <v>1.1399999999999999</v>
-      </c>
-    </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A24">
         <v>2022</v>
       </c>
-      <c r="B24" s="2">
+      <c r="B24" s="1">
         <v>190242</v>
       </c>
-      <c r="C24" s="1">
-        <v>1.18</v>
-      </c>
-    </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
+    </row>
+    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A25">
         <v>2023</v>
       </c>
-      <c r="B25" s="2">
+      <c r="B25" s="1">
         <v>187427</v>
       </c>
-      <c r="C25" s="1">
-        <v>1.44</v>
-      </c>
-    </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
+    </row>
+    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A26">
         <v>2024</v>
       </c>
-      <c r="B26" s="2">
+      <c r="B26" s="1">
         <v>186273</v>
-      </c>
-      <c r="C26" s="1">
-        <v>1.51</v>
       </c>
     </row>
   </sheetData>

</xml_diff>